<commit_message>
Make the target sheet required, not optional (#25)
Per @pearsonca: with the by-target use-case, there is no such thing as a
target-less input -- imurun always predicts coverage for named populations. So
the target sheet/file is now required:

- read_workbook errors if the target sheet is absent (reported alongside any
  other missing required sheets); read_inputs requires target.csv/.rds in
  directory mode (check_all_inputs includes it).
- Docs, the template/example instructions, and the schema drop the "optional"
  framing.
- The corrupt fixture gains a valid target sheet (the corruption is in the
  observations sheet, which is what validation should catch).
- Tests updated: the "omits target when absent" test now asserts an error;
  target-less inputs across the loader/workbook tests gain a target.

Full suite: 121 pass / 0 fail. Spelling clean.
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/example_corrupt.xlsx
+++ b/tests/testthat/fixtures/example_corrupt.xlsx
@@ -10,6 +10,7 @@
     <sheet name="instructions" sheetId="1" r:id="rId1"/>
     <sheet name="observations" sheetId="2" r:id="rId2"/>
     <sheet name="locations" sheetId="3" r:id="rId3"/>
+    <sheet name="target" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +479,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>target sheet -- optional; populations to predict coverage for:</t>
+          <t>target sheet -- the populations to predict coverage for (required):</t>
         </is>
       </c>
     </row>
@@ -17695,4 +17696,77 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Birth cohort</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Youngest age</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Oldest age</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Dose</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Scruggs; Simone</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>31</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>schools, ages 1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Watson</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>